<commit_message>
QoE: dev deal 2 (Tidewell Distribution, NetSuite) with panel-reviewed answer key
16 management adjustments and 3 diligence items; a month missing from the
GL export, a schedule total that does not foot, and dimension noise.
Spec: EXCESS_GL_ACTIVITY carry rule, OUT_OF_PERIOD trigger on any period
label, SIGN_ERROR follows the entries, documented export gaps as
diligence items, and false accepts defined as accepts that overstate EBITDA.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JLUCnhLjHTv59cWHgDLiCw
</commit_message>
<xml_diff>
--- a/qoe-evidence-review/data/dev/tidewell_distribution/adjustments/management_adjusted_ebitda.xlsx
+++ b/qoe-evidence-review/data/dev/tidewell_distribution/adjustments/management_adjusted_ebitda.xlsx
@@ -543,13 +543,13 @@
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="3" t="inlineStr"/>
       <c r="G7" s="5" t="n">
-        <v>6473687.22</v>
+        <v>6472822.83</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>6025143.77</v>
+        <v>5946413.53</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>6185972.12</v>
+        <v>6112732.7</v>
       </c>
     </row>
     <row r="8">
@@ -627,13 +627,13 @@
       <c r="E11" s="6" t="inlineStr"/>
       <c r="F11" s="6" t="inlineStr"/>
       <c r="G11" s="8" t="n">
-        <v>7659096.28</v>
+        <v>7658231.89</v>
       </c>
       <c r="H11" s="8" t="n">
-        <v>7310760.71</v>
+        <v>7232030.47</v>
       </c>
       <c r="I11" s="8" t="n">
-        <v>7517054.01</v>
+        <v>7443814.59</v>
       </c>
     </row>
     <row r="13">
@@ -1321,13 +1321,13 @@
       <c r="E31" s="6" t="inlineStr"/>
       <c r="F31" s="6" t="inlineStr"/>
       <c r="G31" s="8" t="n">
-        <v>8307096.28</v>
+        <v>8306231.89</v>
       </c>
       <c r="H31" s="8" t="n">
-        <v>8703760.710000001</v>
+        <v>8625030.470000001</v>
       </c>
       <c r="I31" s="8" t="n">
-        <v>9045684.189999999</v>
+        <v>8972444.77</v>
       </c>
     </row>
   </sheetData>

</xml_diff>